<commit_message>
Excel: fix DO scan log Acs6 rice hull; note Acs5 Therefore absent in App C
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_009.xlsx
+++ b/thesis/007_CompiledResult_Draft_009.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="B2:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -893,7 +893,6 @@
     <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="72" t="inlineStr">
         <is>
@@ -908,7 +907,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="63" t="inlineStr">
         <is>
@@ -1053,7 +1051,6 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="63" t="inlineStr">
         <is>
@@ -1138,7 +1135,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="63" t="inlineStr">
         <is>
@@ -1491,7 +1487,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="63" t="inlineStr">
         <is>
@@ -1591,7 +1586,6 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="63" t="inlineStr">
         <is>
@@ -1661,7 +1655,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="63" t="inlineStr">
         <is>
@@ -1817,7 +1810,6 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="B63" s="63" t="inlineStr">
         <is>
@@ -1924,7 +1916,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="B72" s="64" t="inlineStr">
         <is>
@@ -1932,7 +1923,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="B74" s="63" t="inlineStr">
         <is>
@@ -12080,7 +12070,7 @@
       </c>
       <c r="E17" s="54" t="inlineStr">
         <is>
-          <t>Therefore, the... (yield inference connector)</t>
+          <t>(Not present in current Appendix C Acs5 text; scan log entry retired for display sync.)</t>
         </is>
       </c>
       <c r="F17" s="54" t="inlineStr">
@@ -12111,7 +12101,7 @@
       <c r="A18" s="49" t="n"/>
       <c r="B18" s="53" t="inlineStr">
         <is>
-          <t>Acs7</t>
+          <t>Acs6</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">

</xml_diff>